<commit_message>
I have updated Monthly budget 01 file
</commit_message>
<xml_diff>
--- a/MonthlyBudget-01.xlsx
+++ b/MonthlyBudget-01.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57de5c48f32aaca3/OfficeNewb/Videos/MicrosoftOffice/Excel101/Exercises/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c-rv90002053\Personal Documents\Ravi\Data\GIT\Sample Data\repo1\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6999D830-5CA0-4B96-A881-CA2FD0C13F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7035"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MONTHLY BUDGET" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -60,12 +72,15 @@
   </si>
   <si>
     <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>Chain EMI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -377,16 +392,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -406,7 +424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -424,11 +442,11 @@
         <v>3600</v>
       </c>
       <c r="F5">
-        <f>E5/$E$10</f>
-        <v>0.61172472387425658</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <f>E5/$E$11</f>
+        <v>0.52439912600145666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -446,11 +464,11 @@
         <v>750</v>
       </c>
       <c r="F6">
-        <f t="shared" ref="F6:F10" si="0">E6/$E$10</f>
-        <v>0.12744265080713679</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <f>E6/$E$11</f>
+        <v>0.10924981791697014</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -468,11 +486,11 @@
         <v>395</v>
       </c>
       <c r="F7">
-        <f t="shared" si="0"/>
-        <v>6.7119796091758707E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <f>E7/$E$11</f>
+        <v>5.7538237436270942E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -490,122 +508,150 @@
         <v>900</v>
       </c>
       <c r="F8">
+        <f>E8/$E$11</f>
+        <v>0.13109978150036417</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>400</v>
+      </c>
+      <c r="C9">
+        <v>350</v>
+      </c>
+      <c r="D9">
+        <v>230</v>
+      </c>
+      <c r="E9">
+        <f>SUM(B9:D9)</f>
+        <v>980</v>
+      </c>
+      <c r="F9">
+        <f>E9/$E$11</f>
+        <v>0.14275309541150766</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>75</v>
+      </c>
+      <c r="C10">
+        <v>75</v>
+      </c>
+      <c r="D10">
+        <v>90</v>
+      </c>
+      <c r="E10">
+        <f t="shared" ref="E10:E11" si="0">SUM(B10:D10)</f>
+        <v>240</v>
+      </c>
+      <c r="F10">
+        <f>E10/$E$11</f>
+        <v>3.4959941733430443E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <f>SUM(B5:B10)</f>
+        <v>2350</v>
+      </c>
+      <c r="C11">
+        <f>SUM(C5:C10)</f>
+        <v>2275</v>
+      </c>
+      <c r="D11">
+        <f>SUM(D5:D10)</f>
+        <v>2240</v>
+      </c>
+      <c r="E11">
         <f t="shared" si="0"/>
-        <v>0.15293118096856415</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9">
+        <v>6865</v>
+      </c>
+      <c r="F11">
+        <f>E11/$E$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <f>MIN(B5:B10)</f>
         <v>75</v>
       </c>
-      <c r="C9">
+      <c r="C13">
+        <f t="shared" ref="C13:E13" si="1">MIN(C5:C10)</f>
         <v>75</v>
       </c>
-      <c r="D9">
+      <c r="D13">
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="E9">
-        <f t="shared" ref="E9:E10" si="1">SUM(B9:D9)</f>
+      <c r="E13">
+        <f t="shared" si="1"/>
         <v>240</v>
       </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>4.0781648258283773E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10">
-        <f>SUM(B5:B9)</f>
-        <v>1950</v>
-      </c>
-      <c r="C10">
-        <f>SUM(C5:C9)</f>
-        <v>1925</v>
-      </c>
-      <c r="D10">
-        <f>SUM(D5:D9)</f>
-        <v>2010</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="1"/>
-        <v>5885</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12">
-        <f>MIN(B5:B9)</f>
-        <v>75</v>
-      </c>
-      <c r="C12">
-        <f t="shared" ref="C12:E12" si="2">MIN(C5:C9)</f>
-        <v>75</v>
-      </c>
-      <c r="D12">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14">
+        <f>MAX(B5:B10)</f>
+        <v>1200</v>
+      </c>
+      <c r="C14">
+        <f t="shared" ref="C14:E14" si="2">MAX(C5:C10)</f>
+        <v>1200</v>
+      </c>
+      <c r="D14">
         <f t="shared" si="2"/>
-        <v>90</v>
-      </c>
-      <c r="E12">
+        <v>1200</v>
+      </c>
+      <c r="E14">
         <f t="shared" si="2"/>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13">
-        <f>MAX(B5:B9)</f>
-        <v>1200</v>
-      </c>
-      <c r="C13">
-        <f t="shared" ref="C13:E13" si="3">MAX(C5:C9)</f>
-        <v>1200</v>
-      </c>
-      <c r="D13">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <f>AVERAGE(B5:B10)</f>
+        <v>391.66666666666669</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:E15" si="3">AVERAGE(C5:C10)</f>
+        <v>379.16666666666669</v>
+      </c>
+      <c r="D15">
         <f t="shared" si="3"/>
-        <v>1200</v>
-      </c>
-      <c r="E13">
+        <v>373.33333333333331</v>
+      </c>
+      <c r="E15">
         <f t="shared" si="3"/>
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14">
-        <f>AVERAGE(B5:B9)</f>
-        <v>390</v>
-      </c>
-      <c r="C14">
-        <f t="shared" ref="C14:E14" si="4">AVERAGE(C5:C9)</f>
-        <v>385</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="4"/>
-        <v>402</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="4"/>
-        <v>1177</v>
+        <v>1144.1666666666667</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7ffb99db-04b0-4879-8e73-d3174e57b086}" enabled="1" method="Standard" siteId="{ec3c7dee-d552-494b-a393-7f941a90b985}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
i have added one more record to Mothly budget file
</commit_message>
<xml_diff>
--- a/MonthlyBudget-01.xlsx
+++ b/MonthlyBudget-01.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c-rv90002053\Personal Documents\Ravi\Data\GIT\Sample Data\repo1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c-rv90002053\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6999D830-5CA0-4B96-A881-CA2FD0C13F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716CBDB0-D1BE-4D2D-8D78-4B1CF332E8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>Chain EMI</t>
+  </si>
+  <si>
+    <t>Mac Book</t>
   </si>
 </sst>
 </file>
@@ -393,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.54296875" customWidth="1"/>
@@ -442,8 +445,8 @@
         <v>3600</v>
       </c>
       <c r="F5">
-        <f>E5/$E$11</f>
-        <v>0.52439912600145666</v>
+        <f t="shared" ref="F5:F12" si="0">E5/$E$12</f>
+        <v>0.46789706264621783</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -464,8 +467,8 @@
         <v>750</v>
       </c>
       <c r="F6">
-        <f>E6/$E$11</f>
-        <v>0.10924981791697014</v>
+        <f t="shared" si="0"/>
+        <v>9.7478554717962046E-2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -486,8 +489,8 @@
         <v>395</v>
       </c>
       <c r="F7">
-        <f>E7/$E$11</f>
-        <v>5.7538237436270942E-2</v>
+        <f t="shared" si="0"/>
+        <v>5.1338705484793343E-2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -508,140 +511,162 @@
         <v>900</v>
       </c>
       <c r="F8">
-        <f>E8/$E$11</f>
-        <v>0.13109978150036417</v>
+        <f t="shared" si="0"/>
+        <v>0.11697426566155446</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="C9">
-        <v>350</v>
+        <v>234</v>
       </c>
       <c r="D9">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="E9">
         <f>SUM(B9:D9)</f>
-        <v>980</v>
+        <v>829</v>
       </c>
       <c r="F9">
-        <f>E9/$E$11</f>
-        <v>0.14275309541150766</v>
+        <f t="shared" si="0"/>
+        <v>0.10774629581492072</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B10">
-        <v>75</v>
+        <v>400</v>
       </c>
       <c r="C10">
-        <v>75</v>
+        <v>350</v>
       </c>
       <c r="D10">
-        <v>90</v>
+        <v>230</v>
       </c>
       <c r="E10">
-        <f t="shared" ref="E10:E11" si="0">SUM(B10:D10)</f>
-        <v>240</v>
+        <f>SUM(B10:D10)</f>
+        <v>980</v>
       </c>
       <c r="F10">
-        <f>E10/$E$11</f>
-        <v>3.4959941733430443E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12737197816480375</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>75</v>
+      </c>
+      <c r="C11">
+        <v>75</v>
+      </c>
+      <c r="D11">
+        <v>90</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ref="E11:E12" si="1">SUM(B11:D11)</f>
+        <v>240</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>3.1193137509747854E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>7</v>
       </c>
-      <c r="B11">
-        <f>SUM(B5:B10)</f>
-        <v>2350</v>
-      </c>
-      <c r="C11">
-        <f>SUM(C5:C10)</f>
-        <v>2275</v>
-      </c>
-      <c r="D11">
-        <f>SUM(D5:D10)</f>
-        <v>2240</v>
-      </c>
-      <c r="E11">
+      <c r="B12">
+        <f>SUM(B5:B11)</f>
+        <v>2700</v>
+      </c>
+      <c r="C12">
+        <f>SUM(C5:C11)</f>
+        <v>2509</v>
+      </c>
+      <c r="D12">
+        <f>SUM(D5:D11)</f>
+        <v>2485</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>7694</v>
+      </c>
+      <c r="F12">
         <f t="shared" si="0"/>
-        <v>6865</v>
-      </c>
-      <c r="F11">
-        <f>E11/$E$11</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13">
-        <f>MIN(B5:B10)</f>
-        <v>75</v>
-      </c>
-      <c r="C13">
-        <f t="shared" ref="C13:E13" si="1">MIN(C5:C10)</f>
-        <v>75</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="1"/>
-        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14">
-        <f>MAX(B5:B10)</f>
-        <v>1200</v>
+        <f>MIN(B5:B11)</f>
+        <v>75</v>
       </c>
       <c r="C14">
-        <f t="shared" ref="C14:E14" si="2">MAX(C5:C10)</f>
-        <v>1200</v>
+        <f t="shared" ref="C14:E14" si="2">MIN(C5:C11)</f>
+        <v>75</v>
       </c>
       <c r="D14">
         <f t="shared" si="2"/>
-        <v>1200</v>
+        <v>90</v>
       </c>
       <c r="E14">
         <f t="shared" si="2"/>
-        <v>3600</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15">
-        <f>AVERAGE(B5:B10)</f>
-        <v>391.66666666666669</v>
+        <f>MAX(B5:B11)</f>
+        <v>1200</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:E15" si="3">AVERAGE(C5:C10)</f>
-        <v>379.16666666666669</v>
+        <f t="shared" ref="C15:E15" si="3">MAX(C5:C11)</f>
+        <v>1200</v>
       </c>
       <c r="D15">
         <f t="shared" si="3"/>
-        <v>373.33333333333331</v>
+        <v>1200</v>
       </c>
       <c r="E15">
         <f t="shared" si="3"/>
-        <v>1144.1666666666667</v>
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <f>AVERAGE(B5:B11)</f>
+        <v>385.71428571428572</v>
+      </c>
+      <c r="C16">
+        <f t="shared" ref="C16:E16" si="4">AVERAGE(C5:C11)</f>
+        <v>358.42857142857144</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="4"/>
+        <v>355</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="4"/>
+        <v>1099.1428571428571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>